<commit_message>
Fixed failed Purchase test scenarios and Updated LOV selection method
Fixed failed Purchase test scenarios and Updated LOV selection method
</commit_message>
<xml_diff>
--- a/testdata/PoToGRN-FOC Scenarios.xlsx
+++ b/testdata/PoToGRN-FOC Scenarios.xlsx
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2586" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2742" uniqueCount="224">
   <si>
     <t>Purchase Order &amp; GRN</t>
   </si>
@@ -572,6 +572,159 @@
   </si>
   <si>
     <t>161.992</t>
+  </si>
+  <si>
+    <t>630</t>
+  </si>
+  <si>
+    <t>6859.72364</t>
+  </si>
+  <si>
+    <t>1118</t>
+  </si>
+  <si>
+    <t>5018.61692</t>
+  </si>
+  <si>
+    <t>2082</t>
+  </si>
+  <si>
+    <t>3679.49017</t>
+  </si>
+  <si>
+    <t>3718</t>
+  </si>
+  <si>
+    <t>2982.50151</t>
+  </si>
+  <si>
+    <t>544</t>
+  </si>
+  <si>
+    <t>2121.79328</t>
+  </si>
+  <si>
+    <t>1783</t>
+  </si>
+  <si>
+    <t>1781.28226</t>
+  </si>
+  <si>
+    <t>4476.1466</t>
+  </si>
+  <si>
+    <t>1272</t>
+  </si>
+  <si>
+    <t>3083.62724</t>
+  </si>
+  <si>
+    <t>545</t>
+  </si>
+  <si>
+    <t>8188.3901</t>
+  </si>
+  <si>
+    <t>1788</t>
+  </si>
+  <si>
+    <t>5322.85475</t>
+  </si>
+  <si>
+    <t>699</t>
+  </si>
+  <si>
+    <t>4538.80752</t>
+  </si>
+  <si>
+    <t>1258</t>
+  </si>
+  <si>
+    <t>3167.55516</t>
+  </si>
+  <si>
+    <t>211.656</t>
+  </si>
+  <si>
+    <t>13748.09797</t>
+  </si>
+  <si>
+    <t>678.991</t>
+  </si>
+  <si>
+    <t>10681.35923</t>
+  </si>
+  <si>
+    <t>533.322</t>
+  </si>
+  <si>
+    <t>7162.62564</t>
+  </si>
+  <si>
+    <t>1540.992</t>
+  </si>
+  <si>
+    <t>5550.52354</t>
+  </si>
+  <si>
+    <t>303.985</t>
+  </si>
+  <si>
+    <t>11450.08032</t>
+  </si>
+  <si>
+    <t>833.326</t>
+  </si>
+  <si>
+    <t>8534.62923</t>
+  </si>
+  <si>
+    <t>475.65</t>
+  </si>
+  <si>
+    <t>11276.18743</t>
+  </si>
+  <si>
+    <t>1146.993</t>
+  </si>
+  <si>
+    <t>7581.88817</t>
+  </si>
+  <si>
+    <t>270.987</t>
+  </si>
+  <si>
+    <t>12627.95556</t>
+  </si>
+  <si>
+    <t>906.658</t>
+  </si>
+  <si>
+    <t>10072.50148</t>
+  </si>
+  <si>
+    <t>467.991</t>
+  </si>
+  <si>
+    <t>9750.1385</t>
+  </si>
+  <si>
+    <t>1086</t>
+  </si>
+  <si>
+    <t>6642.66948</t>
+  </si>
+  <si>
+    <t>463.327</t>
+  </si>
+  <si>
+    <t>8765.64227</t>
+  </si>
+  <si>
+    <t>1599.992</t>
+  </si>
+  <si>
+    <t>7754.44104</t>
   </si>
 </sst>
 </file>
@@ -1715,71 +1868,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="20.5727272727273" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="10" width="5.85454545454545" customWidth="1"/>
-    <col min="11" max="11" width="6" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.2818181818182" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="21" width="9.85454545454546" customWidth="1"/>
-    <col min="22" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="25.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="20.5727272727273"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="10" customWidth="true" width="5.85454545454545"/>
+    <col min="11" max="11" customWidth="true" width="6.0"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.2818181818182"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="10.0"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="21" customWidth="true" width="9.85454545454546"/>
+    <col min="22" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="25.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -2323,11 +2476,11 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="AU4" t="s">
-        <v>79</v>
-      </c>
-      <c r="AV4" t="s">
-        <v>80</v>
+      <c r="AU4" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="AV4" t="s" s="0">
+        <v>174</v>
       </c>
       <c r="AW4" s="35">
         <f>AM4</f>
@@ -2341,7 +2494,7 @@
         <f>AU4+AW4</f>
         <v>4</v>
       </c>
-      <c r="AZ4" t="s">
+      <c r="AZ4" t="s" s="0">
         <v>80</v>
       </c>
       <c r="BA4" s="36"/>
@@ -2366,11 +2519,11 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
-        <v>86</v>
-      </c>
-      <c r="BN4" t="s">
-        <v>87</v>
+      <c r="BM4" t="s" s="0">
+        <v>176</v>
+      </c>
+      <c r="BN4" t="s" s="0">
+        <v>175</v>
       </c>
       <c r="BO4" s="35">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -2529,71 +2682,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="28.2818181818182" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="28.2818181818182"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -3137,6 +3290,8 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
+      <c r="AU4" s="0"/>
+      <c r="AV4" s="0"/>
       <c r="AW4" s="35">
         <f>AM4</f>
         <v>4</v>
@@ -3175,10 +3330,10 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>100</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>100</v>
       </c>
       <c r="BO4" s="35">
@@ -3326,71 +3481,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="24.7181818181818" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="24.7181818181818"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -3934,11 +4089,11 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="AU4" t="s">
-        <v>118</v>
-      </c>
-      <c r="AV4" t="s">
-        <v>119</v>
+      <c r="AU4" t="s" s="0">
+        <v>188</v>
+      </c>
+      <c r="AV4" t="s" s="0">
+        <v>189</v>
       </c>
       <c r="AW4" s="35">
         <f>AM4</f>
@@ -3978,11 +4133,11 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
-        <v>120</v>
-      </c>
-      <c r="BN4" t="s">
-        <v>121</v>
+      <c r="BM4" t="s" s="0">
+        <v>191</v>
+      </c>
+      <c r="BN4" t="s" s="0">
+        <v>190</v>
       </c>
       <c r="BO4" s="35">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -4141,71 +4296,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="24.7181818181818" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="24.7181818181818"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -4749,11 +4904,11 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="AU4" t="s">
-        <v>123</v>
-      </c>
-      <c r="AV4" t="s">
-        <v>124</v>
+      <c r="AU4" t="s" s="0">
+        <v>192</v>
+      </c>
+      <c r="AV4" t="s" s="0">
+        <v>193</v>
       </c>
       <c r="AW4" s="35">
         <f>AM4</f>
@@ -4793,11 +4948,11 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
-        <v>125</v>
-      </c>
-      <c r="BN4" t="s">
-        <v>126</v>
+      <c r="BM4" t="s" s="0">
+        <v>195</v>
+      </c>
+      <c r="BN4" t="s" s="0">
+        <v>194</v>
       </c>
       <c r="BO4" s="35">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -4944,71 +5099,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="25.1454545454545" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="25.1454545454545"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -5743,71 +5898,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="22.0"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -6351,6 +6506,8 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
+      <c r="AU4" s="0"/>
+      <c r="AV4" s="0"/>
       <c r="AW4" s="35">
         <f>AM4</f>
         <v>4</v>
@@ -6389,10 +6546,10 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>100</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>100</v>
       </c>
       <c r="BO4" s="35">
@@ -6540,71 +6697,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="22.0"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -7148,6 +7305,8 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
+      <c r="AU4" s="0"/>
+      <c r="AV4" s="0"/>
       <c r="AW4" s="35">
         <f>AM4</f>
         <v>4</v>
@@ -7186,10 +7345,10 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>100</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>100</v>
       </c>
       <c r="BO4" s="35">
@@ -7337,71 +7496,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="24.5727272727273" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="24.5727272727273"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -7945,11 +8104,11 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="AU4" t="s">
-        <v>131</v>
-      </c>
-      <c r="AV4" t="s">
-        <v>132</v>
+      <c r="AU4" t="s" s="0">
+        <v>196</v>
+      </c>
+      <c r="AV4" t="s" s="0">
+        <v>197</v>
       </c>
       <c r="AW4" s="35">
         <f>AM4</f>
@@ -7963,7 +8122,7 @@
         <f>AU4+AW4</f>
         <v>32.6603333333333</v>
       </c>
-      <c r="AZ4" t="s">
+      <c r="AZ4" t="s" s="0">
         <v>132</v>
       </c>
       <c r="BA4" s="36"/>
@@ -7988,11 +8147,11 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
-        <v>133</v>
-      </c>
-      <c r="BN4" t="s">
-        <v>134</v>
+      <c r="BM4" t="s" s="0">
+        <v>199</v>
+      </c>
+      <c r="BN4" t="s" s="0">
+        <v>198</v>
       </c>
       <c r="BO4" s="35">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -8151,71 +8310,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="24.5727272727273" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="24.5727272727273"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -8759,11 +8918,11 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="AU4" t="s">
-        <v>136</v>
-      </c>
-      <c r="AV4" t="s">
-        <v>137</v>
+      <c r="AU4" t="s" s="0">
+        <v>200</v>
+      </c>
+      <c r="AV4" t="s" s="0">
+        <v>201</v>
       </c>
       <c r="AW4" s="35">
         <f>AM4</f>
@@ -8777,7 +8936,7 @@
         <f>AU4+AW4</f>
         <v>83.3283333333333</v>
       </c>
-      <c r="AZ4" t="s">
+      <c r="AZ4" t="s" s="0">
         <v>137</v>
       </c>
       <c r="BA4" s="36"/>
@@ -8802,11 +8961,11 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
-        <v>138</v>
-      </c>
-      <c r="BN4" t="s">
-        <v>139</v>
+      <c r="BM4" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="BN4" t="s" s="0">
+        <v>202</v>
       </c>
       <c r="BO4" s="35">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -8965,71 +9124,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="22.0"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -9573,6 +9732,8 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
+      <c r="AU4" s="0"/>
+      <c r="AV4" s="0"/>
       <c r="AW4" s="35">
         <f>AM4</f>
         <v>4</v>
@@ -9611,10 +9772,10 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>100</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>100</v>
       </c>
       <c r="BO4" s="35">
@@ -9762,71 +9923,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="22.0"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -10370,6 +10531,8 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
+      <c r="AU4" s="0"/>
+      <c r="AV4" s="0"/>
       <c r="AW4" s="35">
         <f>AM4</f>
         <v>4</v>
@@ -10408,10 +10571,10 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>100</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>100</v>
       </c>
       <c r="BO4" s="35">
@@ -10559,72 +10722,72 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="2" width="21.8545454545455" customWidth="1"/>
-    <col min="3" max="3" width="27.5727272727273" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="10" width="5.85454545454545" customWidth="1"/>
-    <col min="11" max="11" width="6" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.2818181818182" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="21" width="9.85454545454546" customWidth="1"/>
-    <col min="22" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="25.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="2" customWidth="true" width="21.8545454545455"/>
+    <col min="3" max="3" customWidth="true" width="27.5727272727273"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="10" customWidth="true" width="5.85454545454545"/>
+    <col min="11" max="11" customWidth="true" width="6.0"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.2818181818182"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="10.0"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="21" customWidth="true" width="9.85454545454546"/>
+    <col min="22" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="25.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -11168,11 +11331,11 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="AU4" t="s">
-        <v>91</v>
-      </c>
-      <c r="AV4" t="s">
-        <v>92</v>
+      <c r="AU4" t="s" s="0">
+        <v>177</v>
+      </c>
+      <c r="AV4" t="s" s="0">
+        <v>178</v>
       </c>
       <c r="AW4" s="35">
         <f>AM4</f>
@@ -11186,7 +11349,7 @@
         <f>AU4+AW4</f>
         <v>4</v>
       </c>
-      <c r="AZ4" t="s">
+      <c r="AZ4" t="s" s="0">
         <v>92</v>
       </c>
       <c r="BA4" s="36"/>
@@ -11211,11 +11374,11 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
-        <v>93</v>
-      </c>
-      <c r="BN4" t="s">
-        <v>94</v>
+      <c r="BM4" t="s" s="0">
+        <v>180</v>
+      </c>
+      <c r="BN4" t="s" s="0">
+        <v>179</v>
       </c>
       <c r="BO4" s="35">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -11362,71 +11525,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="28.0"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -11970,11 +12133,11 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="AU4" t="s">
-        <v>143</v>
-      </c>
-      <c r="AV4" t="s">
-        <v>144</v>
+      <c r="AU4" t="s" s="0">
+        <v>204</v>
+      </c>
+      <c r="AV4" t="s" s="0">
+        <v>205</v>
       </c>
       <c r="AW4" s="35">
         <f>AM4</f>
@@ -12014,11 +12177,11 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
-        <v>145</v>
-      </c>
-      <c r="BN4" t="s">
-        <v>146</v>
+      <c r="BM4" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="BN4" t="s" s="0">
+        <v>206</v>
       </c>
       <c r="BO4" s="35">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -12177,71 +12340,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="28.0"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -12785,11 +12948,11 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="AU4" t="s">
-        <v>148</v>
-      </c>
-      <c r="AV4" t="s">
-        <v>149</v>
+      <c r="AU4" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="AV4" t="s" s="0">
+        <v>209</v>
       </c>
       <c r="AW4" s="35">
         <f>AM4</f>
@@ -12829,11 +12992,11 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
-        <v>150</v>
-      </c>
-      <c r="BN4" t="s">
-        <v>151</v>
+      <c r="BM4" t="s" s="0">
+        <v>211</v>
+      </c>
+      <c r="BN4" t="s" s="0">
+        <v>210</v>
       </c>
       <c r="BO4" s="35">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -12992,71 +13155,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="28.0"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -13600,11 +13763,11 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="AU4" t="s">
-        <v>152</v>
-      </c>
-      <c r="AV4" t="s">
-        <v>153</v>
+      <c r="AU4" t="s" s="0">
+        <v>204</v>
+      </c>
+      <c r="AV4" t="s" s="0">
+        <v>205</v>
       </c>
       <c r="AW4" s="35">
         <f>AM4</f>
@@ -13644,11 +13807,11 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
-        <v>145</v>
-      </c>
-      <c r="BN4" t="s">
-        <v>146</v>
+      <c r="BM4" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="BN4" t="s" s="0">
+        <v>206</v>
       </c>
       <c r="BO4" s="35">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -13795,71 +13958,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="28.0"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -14403,11 +14566,11 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="AU4" t="s">
-        <v>154</v>
-      </c>
-      <c r="AV4" t="s">
-        <v>155</v>
+      <c r="AU4" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="AV4" t="s" s="0">
+        <v>209</v>
       </c>
       <c r="AW4" s="35">
         <f>AM4</f>
@@ -14447,11 +14610,11 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
-        <v>150</v>
-      </c>
-      <c r="BN4" t="s">
-        <v>151</v>
+      <c r="BM4" t="s" s="0">
+        <v>211</v>
+      </c>
+      <c r="BN4" t="s" s="0">
+        <v>210</v>
       </c>
       <c r="BO4" s="35">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -14598,71 +14761,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="27.5727272727273" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="27.5727272727273"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -15206,11 +15369,11 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="AU4" t="s">
-        <v>157</v>
-      </c>
-      <c r="AV4" t="s">
-        <v>158</v>
+      <c r="AU4" t="s" s="0">
+        <v>212</v>
+      </c>
+      <c r="AV4" t="s" s="0">
+        <v>213</v>
       </c>
       <c r="AW4" s="35">
         <f>AM4</f>
@@ -15250,11 +15413,11 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
-        <v>159</v>
-      </c>
-      <c r="BN4" t="s">
-        <v>160</v>
+      <c r="BM4" t="s" s="0">
+        <v>215</v>
+      </c>
+      <c r="BN4" t="s" s="0">
+        <v>214</v>
       </c>
       <c r="BO4" s="35">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -15413,71 +15576,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="27.5727272727273" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="27.5727272727273"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -16021,11 +16184,11 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="AU4" t="s">
-        <v>162</v>
-      </c>
-      <c r="AV4" t="s">
-        <v>163</v>
+      <c r="AU4" t="s" s="0">
+        <v>216</v>
+      </c>
+      <c r="AV4" t="s" s="0">
+        <v>217</v>
       </c>
       <c r="AW4" s="35">
         <f>AM4</f>
@@ -16065,11 +16228,11 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
-        <v>164</v>
-      </c>
-      <c r="BN4" t="s">
-        <v>165</v>
+      <c r="BM4" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="BN4" t="s" s="0">
+        <v>218</v>
       </c>
       <c r="BO4" s="35">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -16228,71 +16391,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="27.5727272727273" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="27.5727272727273"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -16836,11 +16999,11 @@
       <c r="AT4" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="AU4" t="s">
-        <v>166</v>
-      </c>
-      <c r="AV4" t="s">
-        <v>167</v>
+      <c r="AU4" t="s" s="0">
+        <v>212</v>
+      </c>
+      <c r="AV4" t="s" s="0">
+        <v>213</v>
       </c>
       <c r="AW4" s="16">
         <f>AM4</f>
@@ -16880,11 +17043,11 @@
       <c r="BL4" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
-        <v>159</v>
-      </c>
-      <c r="BN4" t="s">
-        <v>160</v>
+      <c r="BM4" t="s" s="0">
+        <v>215</v>
+      </c>
+      <c r="BN4" t="s" s="0">
+        <v>214</v>
       </c>
       <c r="BO4" s="16">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -17031,71 +17194,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="27.5727272727273" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="27.5727272727273"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -17639,11 +17802,11 @@
       <c r="AT4" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="AU4" t="s">
-        <v>169</v>
-      </c>
-      <c r="AV4" t="s">
-        <v>170</v>
+      <c r="AU4" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="AV4" t="s" s="0">
+        <v>221</v>
       </c>
       <c r="AW4" s="16">
         <f>AM4</f>
@@ -17683,11 +17846,11 @@
       <c r="BL4" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
-        <v>171</v>
-      </c>
-      <c r="BN4" t="s">
-        <v>172</v>
+      <c r="BM4" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="BN4" t="s" s="0">
+        <v>222</v>
       </c>
       <c r="BO4" s="16">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -17834,71 +17997,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="22.0"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -18633,71 +18796,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="25.0"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -19241,6 +19404,8 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
+      <c r="AU4" s="0"/>
+      <c r="AV4" s="0"/>
       <c r="AW4" s="35">
         <f>AM4</f>
         <v>4</v>
@@ -19279,10 +19444,10 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>100</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>100</v>
       </c>
       <c r="BO4" s="35">
@@ -19430,71 +19595,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="25.0"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -20038,6 +20203,8 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
+      <c r="AU4" s="0"/>
+      <c r="AV4" s="0"/>
       <c r="AW4" s="35">
         <f>AM4</f>
         <v>4</v>
@@ -20076,10 +20243,10 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>100</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>100</v>
       </c>
       <c r="BO4" s="35">
@@ -20227,71 +20394,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="25.2818181818182" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="25.2818181818182"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -20835,11 +21002,11 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="AU4" t="s">
-        <v>105</v>
-      </c>
-      <c r="AV4" t="s">
-        <v>106</v>
+      <c r="AU4" t="s" s="0">
+        <v>181</v>
+      </c>
+      <c r="AV4" t="s" s="0">
+        <v>182</v>
       </c>
       <c r="AW4" s="35">
         <f>AM4</f>
@@ -20879,11 +21046,11 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
-        <v>107</v>
-      </c>
-      <c r="BN4" t="s">
-        <v>108</v>
+      <c r="BM4" t="s" s="0">
+        <v>184</v>
+      </c>
+      <c r="BN4" t="s" s="0">
+        <v>183</v>
       </c>
       <c r="BO4" s="35">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -21042,71 +21209,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="25.2818181818182" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="25.2818181818182"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -21650,11 +21817,11 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="AU4" t="s">
-        <v>110</v>
-      </c>
-      <c r="AV4" t="s">
-        <v>111</v>
+      <c r="AU4" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="AV4" t="s" s="0">
+        <v>185</v>
       </c>
       <c r="AW4" s="35">
         <f>AM4</f>
@@ -21694,11 +21861,11 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
-        <v>112</v>
-      </c>
-      <c r="BN4" t="s">
-        <v>113</v>
+      <c r="BM4" t="s" s="0">
+        <v>187</v>
+      </c>
+      <c r="BN4" t="s" s="0">
+        <v>186</v>
       </c>
       <c r="BO4" s="35">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -21845,71 +22012,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="25.5727272727273" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="25.5727272727273"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -22644,71 +22811,71 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="5.14545454545455" customWidth="1"/>
-    <col min="2" max="3" width="28.2818181818182" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="5.14545454545455" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="10" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="10" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="5.14545454545455"/>
+    <col min="2" max="3" customWidth="true" width="28.2818181818182"/>
+    <col min="4" max="4" customWidth="true" width="79.4272727272727"/>
+    <col min="5" max="5" customWidth="true" width="11.5727272727273"/>
+    <col min="6" max="6" customWidth="true" width="5.14545454545455"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7181818181818"/>
+    <col min="9" max="9" customWidth="true" width="5.85454545454545"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85454545454545"/>
+    <col min="12" max="12" customWidth="true" width="14.2818181818182"/>
+    <col min="13" max="13" customWidth="true" width="9.42727272727273"/>
+    <col min="14" max="14" customWidth="true" width="14.4272727272727"/>
+    <col min="15" max="15" customWidth="true" width="15.5727272727273"/>
+    <col min="16" max="16" customWidth="true" width="14.4272727272727"/>
+    <col min="17" max="17" customWidth="true" width="39.4272727272727"/>
+    <col min="18" max="18" customWidth="true" width="11.7181818181818"/>
+    <col min="19" max="19" customWidth="true" width="11.8545454545455"/>
+    <col min="20" max="20" customWidth="true" width="6.42727272727273"/>
+    <col min="21" max="22" customWidth="true" width="6.57272727272727"/>
+    <col min="23" max="23" customWidth="true" width="37.1454545454545"/>
+    <col min="24" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71818181818182"/>
+    <col min="27" max="27" customWidth="true" width="6.28181818181818"/>
+    <col min="28" max="28" customWidth="true" width="9.28181818181818"/>
+    <col min="29" max="29" customWidth="true" width="9.71818181818182"/>
+    <col min="30" max="30" customWidth="true" width="12.8545454545455"/>
+    <col min="31" max="31" customWidth="true" width="16.1454545454545"/>
+    <col min="32" max="32" customWidth="true" width="15.4272727272727"/>
+    <col min="33" max="33" customWidth="true" width="24.5727272727273"/>
+    <col min="34" max="34" customWidth="true" width="8.57272727272727"/>
+    <col min="35" max="35" customWidth="true" width="14.7181818181818"/>
+    <col min="36" max="36" customWidth="true" width="18.5727272727273"/>
+    <col min="37" max="37" customWidth="true" width="14.1454545454545"/>
+    <col min="38" max="38" customWidth="true" width="14.7181818181818"/>
+    <col min="39" max="39" customWidth="true" width="17.4272727272727"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5727272727273"/>
+    <col min="42" max="42" customWidth="true" width="25.2818181818182"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7181818181818"/>
+    <col min="45" max="45" customWidth="true" width="10.0"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5727272727273"/>
+    <col min="48" max="48" customWidth="true" width="21.1454545454545"/>
+    <col min="49" max="49" customWidth="true" width="11.5727272727273"/>
+    <col min="50" max="50" customWidth="true" width="16.7181818181818"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4272727272727"/>
+    <col min="53" max="53" customWidth="true" width="18.8545454545455"/>
+    <col min="54" max="54" customWidth="true" width="23.2818181818182"/>
+    <col min="55" max="55" customWidth="true" width="15.5727272727273"/>
+    <col min="56" max="56" customWidth="true" width="14.2818181818182"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2818181818182"/>
+    <col min="59" max="59" customWidth="true" width="13.5727272727273"/>
+    <col min="60" max="61" customWidth="true" width="12.7181818181818"/>
+    <col min="62" max="62" customWidth="true" width="21.8545454545455"/>
+    <col min="63" max="63" customWidth="true" width="30.5727272727273"/>
+    <col min="64" max="64" customWidth="true" width="10.0"/>
+    <col min="65" max="65" customWidth="true" width="42.5727272727273"/>
+    <col min="66" max="66" customWidth="true" width="38.1454545454545"/>
+    <col min="67" max="67" customWidth="true" width="19.4272727272727"/>
+    <col min="68" max="68" customWidth="true" width="35.4272727272727"/>
+    <col min="69" max="69" customWidth="true" width="9.57272727272727"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -23252,6 +23419,8 @@
       <c r="AT4" s="35" t="s">
         <v>76</v>
       </c>
+      <c r="AU4" s="0"/>
+      <c r="AV4" s="0"/>
       <c r="AW4" s="35">
         <f>AM4</f>
         <v>4</v>
@@ -23290,10 +23459,10 @@
       <c r="BL4" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BM4" t="s" s="0">
         <v>100</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BN4" t="s" s="0">
         <v>100</v>
       </c>
       <c r="BO4" s="35">

</xml_diff>